<commit_message>
Frame deck for pre-filing IPR committee approval
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/deliverables/IITBBS_Crash_Barrier_Presentation_Data.xlsx
+++ b/deliverables/IITBBS_Crash_Barrier_Presentation_Data.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="43" customWidth="1" min="1" max="1"/>
@@ -481,10 +481,22 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Patent status</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Not yet filed; presentation prepared for IIT Bhubaneswar IPR committee pre-filing evaluation and approval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
           <t>Generated</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>13 August 2026</t>
         </is>

</xml_diff>

<commit_message>
Restyle patent decks as academic research presentations
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/deliverables/IITBBS_Crash_Barrier_Presentation_Data.xlsx
+++ b/deliverables/IITBBS_Crash_Barrier_Presentation_Data.xlsx
@@ -47,7 +47,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="0008243A"/>
+        <fgColor rgb="0017365D"/>
       </patternFill>
     </fill>
   </fills>
@@ -498,7 +498,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>13 August 2026</t>
+          <t>14 August 2026</t>
         </is>
       </c>
     </row>

</xml_diff>